<commit_message>
alterações no front e back
</commit_message>
<xml_diff>
--- a/squad1/ciento/api-cientometria/Consolidado - Respostas Gerais.xlsx
+++ b/squad1/ciento/api-cientometria/Consolidado - Respostas Gerais.xlsx
@@ -8702,7 +8702,7 @@
         <v>0</v>
       </c>
       <c r="AJ119" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>MANEJO DE NUTRIENTES E AGUA</v>
       </c>
     </row>
     <row r="120">
@@ -8713,94 +8713,94 @@
         <v>izaias silva</v>
       </c>
       <c r="C120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="D120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="E120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="F120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="G120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="H120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="I120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="J120" t="str">
-        <v/>
+        <v>Prova de Administração</v>
       </c>
       <c r="K120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="L120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="M120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="N120" t="str">
-        <v/>
+        <v>Questões discursivas e objetivas</v>
       </c>
       <c r="O120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="P120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="Q120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="R120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="S120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="T120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="U120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="V120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="W120" t="str">
         <v>administracao - silvania silva.pdf</v>
       </c>
       <c r="Z120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="AA120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="AB120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="AC120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="AD120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="AE120" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="AF120" t="str">
-        <v>Rejeitado: O texto não trata de agronomia prática.</v>
-      </c>
-      <c r="AG120" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="AH120" t="str">
-        <v>TRUE</v>
+        <v>N/A</v>
+      </c>
+      <c r="AG120" t="b">
+        <v>0</v>
+      </c>
+      <c r="AH120" t="b">
+        <v>1</v>
       </c>
       <c r="AI120" t="b">
         <v>0</v>
@@ -8905,59 +8905,62 @@
       </c>
     </row>
     <row r="122">
+      <c r="A122">
+        <v>12</v>
+      </c>
       <c r="C122" t="str">
-        <v>Rajinder Pal, Onkar Singh, Gulzar S Sanghera, R K Gupta</v>
+        <v>N/A</v>
       </c>
       <c r="D122" t="str">
-        <v>Influence of INM on sugarcane productivity and soil fertility under Indo-Gangetic plain</v>
+        <v>N/A</v>
       </c>
       <c r="E122" t="str">
-        <v>Desenvolvimento de estratégias de manejo integrado de nutrientes para o cultivo de cana-de-açúcar em condições subtropicais do Punjab</v>
-      </c>
-      <c r="F122">
-        <v>2021</v>
+        <v>N/A</v>
+      </c>
+      <c r="F122" t="str">
+        <v>N/A</v>
       </c>
       <c r="G122" t="str">
         <v>N/A</v>
       </c>
       <c r="H122" t="str">
-        <v>Cana-de-açúcar, Manejo integrado de nutrientes, Fertilidade do solo, Produtividade</v>
+        <v>N/A</v>
       </c>
       <c r="I122" t="str">
-        <v>O estudo teve como objetivo desenvolver estratégias de manejo integrado de nutrientes para o cultivo de cana-de-açúcar em condições subtropicais do Punjab.</v>
+        <v>N/A</v>
       </c>
       <c r="J122" t="str">
-        <v>Artigo científico</v>
+        <v>N/A</v>
       </c>
       <c r="K122" t="str">
-        <v>Indian Journal of Agricultural Sciences</v>
+        <v>N/A</v>
       </c>
       <c r="L122" t="str">
-        <v>Punjab Agricultural University</v>
+        <v>N/A</v>
       </c>
       <c r="M122" t="str">
-        <v>Kapurthala, Punjab, Índia</v>
+        <v>N/A</v>
       </c>
       <c r="N122" t="str">
-        <v>Pesquisa experimental</v>
+        <v>N/A</v>
       </c>
       <c r="O122" t="str">
-        <v>Indian Journal of Agricultural Sciences</v>
+        <v>N/A</v>
       </c>
       <c r="P122" t="str">
         <v>N/A</v>
       </c>
-      <c r="Q122">
-        <v>91</v>
-      </c>
-      <c r="R122">
-        <v>5</v>
+      <c r="Q122" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="R122" t="str">
+        <v>N/A</v>
       </c>
       <c r="S122" t="str">
-        <v>703-707</v>
+        <v>N/A</v>
       </c>
       <c r="T122" t="str">
-        <v>https://doi.org/10.56093/ijas.v91i5.112987</v>
+        <v>N/A</v>
       </c>
       <c r="U122" t="str">
         <v>N/A</v>
@@ -8966,7 +8969,7 @@
         <v>N/A</v>
       </c>
       <c r="W122" t="str">
-        <v>Influence of INM on sugarcane productivity_bioinsumos(1).pdf</v>
+        <v/>
       </c>
       <c r="Z122" t="str">
         <v>N/A</v>
@@ -8987,16 +8990,16 @@
         <v>N/A</v>
       </c>
       <c r="AF122" t="str">
-        <v>Aprovado: Avalia a eficácia de diferentes estratégias de manejo integrado de nutrientes para o cultivo de cana-de-açúcar em condições subtropicais do Punjab.</v>
+        <v>Rejeitado: Texto insuficiente para análise científica.</v>
       </c>
       <c r="AG122" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH122" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ122" t="str">
-        <v>BIOINSUMOS</v>
+        <v>ERRO: PDF sem texto (Imagem/Scan)</v>
       </c>
     </row>
     <row r="123">
@@ -9007,16 +9010,19 @@
         <v>Influence of INM on sugarcane productivity and soil fertility under Indo-Gangetic plain</v>
       </c>
       <c r="E123" t="str">
-        <v>A field experiment was conducted during 2016-17 at Punjab Agricultural University, Regional Research Station, Kapurthala, Punjab, India with nine treatments comprising various combinations of farmyard manure (FYM), bio- fertilizers and different levels of chemical fertilizers in a randomized block design (RBD).</v>
+        <v>Desenvolvimento de estratégias de manejo integrado de nutrientes para o cultivo de cana-de-açúcar em condições subtropicais do Punjab</v>
       </c>
       <c r="F123">
         <v>2021</v>
       </c>
+      <c r="G123" t="str">
+        <v>N/A</v>
+      </c>
       <c r="H123" t="str">
-        <v>Cane and sugar productivity, Integrated nutrient management, Nutrient status, Sugarcane</v>
+        <v>Cana-de-açúcar, Manejo integrado de nutrientes, Fertilidade do solo, Produtividade</v>
       </c>
       <c r="I123" t="str">
-        <v>O estudo teve como objetivo desenvolver estratégias de manejo integrado de nutrientes (INM) para o uso conjuntivo de fontes orgânicas e inorgânicas de nutrientes, além de biofertilizantes, de forma a sustentar a saúde do solo e a produtividade do cana-de-açúcar a longo prazo em condições subtropicais do Punjab.</v>
+        <v>O estudo teve como objetivo desenvolver estratégias de manejo integrado de nutrientes para o cultivo de cana-de-açúcar em condições subtropicais do Punjab.</v>
       </c>
       <c r="J123" t="str">
         <v>Artigo científico</v>
@@ -9031,43 +9037,55 @@
         <v>Kapurthala, Punjab, Índia</v>
       </c>
       <c r="N123" t="str">
-        <v>Experimento de campo</v>
+        <v>Pesquisa experimental</v>
       </c>
       <c r="O123" t="str">
         <v>Indian Journal of Agricultural Sciences</v>
       </c>
+      <c r="P123" t="str">
+        <v>N/A</v>
+      </c>
       <c r="Q123">
         <v>91</v>
       </c>
       <c r="R123">
         <v>5</v>
       </c>
+      <c r="S123" t="str">
+        <v>703-707</v>
+      </c>
       <c r="T123" t="str">
         <v>https://doi.org/10.56093/ijas.v91i5.112987</v>
       </c>
+      <c r="U123" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="V123" t="str">
+        <v>N/A</v>
+      </c>
       <c r="W123" t="str">
         <v>Influence of INM on sugarcane productivity_bioinsumos(1).pdf</v>
       </c>
       <c r="Z123" t="str">
-        <v>O solo da área experimental é um solo arenoso-looso, com pH 8,05, baixo em carbono orgânico (3,70 g/kg) e condutividade elétrica (0,231 dS/m).</v>
+        <v>N/A</v>
       </c>
       <c r="AA123" t="str">
-        <v>Cromatografia gasosa, Espectrometria de massa, Análise de variância (ANOVA)</v>
+        <v>N/A</v>
       </c>
       <c r="AB123" t="str">
-        <v>Nitrogênio, Fósforo, Potássio, Sulfeto de hidrogênio, Ferro, Manganês, Zinco, Cobre</v>
+        <v>N/A</v>
       </c>
       <c r="AC123" t="str">
-        <v>Fertilização de cobertura, Adubação foliar, Fertirrigação</v>
+        <v>N/A</v>
       </c>
       <c r="AD123" t="str">
-        <v>Cana-de-açúcar</v>
+        <v>N/A</v>
       </c>
       <c r="AE123" t="str">
-        <v>Cana-de-açúcar (Saccharum officinarum)</v>
+        <v>N/A</v>
       </c>
       <c r="AF123" t="str">
-        <v>Aprovado: Detalha uma nova estratégia de manejo integrado de nutrientes para cana-de-açúcar.</v>
+        <v>Aprovado: Avalia a eficácia de diferentes estratégias de manejo integrado de nutrientes para o cultivo de cana-de-açúcar em condições subtropicais do Punjab.</v>
       </c>
       <c r="AG123" t="b">
         <v>1</v>
@@ -9081,88 +9099,73 @@
     </row>
     <row r="124">
       <c r="C124" t="str">
-        <v>M.P. Stephan, M. Oliveira, K.R.S. Teixeira, G. Martinez-Drets e J. D/Sbereiner</v>
+        <v>Rajinder Pal, Onkar Singh, Gulzar S Sanghera, R K Gupta</v>
       </c>
       <c r="D124" t="str">
-        <v>Physiology and dinitrogen fixation of A cetobacter diazotrophicus</v>
+        <v>Influence of INM on sugarcane productivity and soil fertility under Indo-Gangetic plain</v>
       </c>
       <c r="E124" t="str">
-        <v>N2-dependent growth; N2-fixation, in sugar cane; Acetobacter diazotrophicus</v>
+        <v>A field experiment was conducted during 2016-17 at Punjab Agricultural University, Regional Research Station, Kapurthala, Punjab, India with nine treatments comprising various combinations of farmyard manure (FYM), bio- fertilizers and different levels of chemical fertilizers in a randomized block design (RBD).</v>
       </c>
       <c r="F124">
-        <v>1991</v>
-      </c>
-      <c r="G124" t="str">
-        <v>N/A</v>
+        <v>2021</v>
       </c>
       <c r="H124" t="str">
-        <v>N2-dependent growth, N2-fixation, sugar cane, Acetobacter diazotrophicus</v>
+        <v>Cane and sugar productivity, Integrated nutrient management, Nutrient status, Sugarcane</v>
       </c>
       <c r="I124" t="str">
-        <v>O artigo descreve as características fisiológicas de Acetobacter diazotrophicus, um diazotrófico isolado de raízes de cana-de-açúcar. O bactério é capaz de crescer em pH 3,0 e apresenta alta atividade de nitrogenase até pH 2,5. A extração de oxidação de glicose seguida pela formação de ácido gluconico é necessária para iniciar o crescimento logarítmico, que ocorre com N2 como fonte de nitrogênio.</v>
+        <v>O estudo teve como objetivo desenvolver estratégias de manejo integrado de nutrientes (INM) para o uso conjuntivo de fontes orgânicas e inorgânicas de nutrientes, além de biofertilizantes, de forma a sustentar a saúde do solo e a produtividade do cana-de-açúcar a longo prazo em condições subtropicais do Punjab.</v>
       </c>
       <c r="J124" t="str">
         <v>Artigo científico</v>
       </c>
       <c r="K124" t="str">
-        <v>FEMS Microbiology Letters</v>
+        <v>Indian Journal of Agricultural Sciences</v>
       </c>
       <c r="L124" t="str">
-        <v>CNPBS/EMBRAPA</v>
+        <v>Punjab Agricultural University</v>
       </c>
       <c r="M124" t="str">
-        <v>Seropédica, Rio de Janeiro, Brasil</v>
+        <v>Kapurthala, Punjab, Índia</v>
       </c>
       <c r="N124" t="str">
-        <v>Estudo de caso</v>
+        <v>Experimento de campo</v>
       </c>
       <c r="O124" t="str">
-        <v>FEMS Microbiology Letters</v>
-      </c>
-      <c r="P124" t="str">
-        <v>N/A</v>
+        <v>Indian Journal of Agricultural Sciences</v>
       </c>
       <c r="Q124">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="R124">
-        <v>1</v>
-      </c>
-      <c r="S124" t="str">
-        <v>67-72</v>
+        <v>5</v>
       </c>
       <c r="T124" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="U124" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="V124" t="str">
-        <v>N/A</v>
+        <v>https://doi.org/10.56093/ijas.v91i5.112987</v>
       </c>
       <c r="W124" t="str">
-        <v>Physiology and dinitrogen fixation of A cetobacter diazotrophicus_bioinsumos.pdf</v>
+        <v>Influence of INM on sugarcane productivity_bioinsumos(1).pdf</v>
       </c>
       <c r="Z124" t="str">
-        <v>O solo da região de cultivo da cana-de-açúcar é caracterizado por pH ácido, com valores entre 3,0 e 5,5. A região é localizada no Brasil, mais especificamente no estado do Rio de Janeiro.</v>
+        <v>O solo da área experimental é um solo arenoso-looso, com pH 8,05, baixo em carbono orgânico (3,70 g/kg) e condutividade elétrica (0,231 dS/m).</v>
       </c>
       <c r="AA124" t="str">
         <v>Cromatografia gasosa, Espectrometria de massa, Análise de variância (ANOVA)</v>
       </c>
       <c r="AB124" t="str">
-        <v>Nitrogênio, Fósforo, Potássio</v>
+        <v>Nitrogênio, Fósforo, Potássio, Sulfeto de hidrogênio, Ferro, Manganês, Zinco, Cobre</v>
       </c>
       <c r="AC124" t="str">
         <v>Fertilização de cobertura, Adubação foliar, Fertirrigação</v>
       </c>
       <c r="AD124" t="str">
-        <v>Cereais, Leguminosas, Hortaliças, Frutíferas</v>
+        <v>Cana-de-açúcar</v>
       </c>
       <c r="AE124" t="str">
-        <v>Cana-de-açúcar</v>
+        <v>Cana-de-açúcar (Saccharum officinarum)</v>
       </c>
       <c r="AF124" t="str">
-        <v>Aprovado: Detalha as características fisiológicas de Acetobacter diazotrophicus e sua capacidade de fixação de nitrogênio.</v>
+        <v>Aprovado: Detalha uma nova estratégia de manejo integrado de nutrientes para cana-de-açúcar.</v>
       </c>
       <c r="AG124" t="b">
         <v>1</v>
@@ -9176,55 +9179,55 @@
     </row>
     <row r="125">
       <c r="C125" t="str">
-        <v>N. SenthiP, T. Raguchander, R. Viswanathan e R. Samiyappan</v>
+        <v>M.P. Stephan, M. Oliveira, K.R.S. Teixeira, G. Martinez-Drets e J. D/Sbereiner</v>
       </c>
       <c r="D125" t="str">
-        <v>Sugarcane Talc Formulated. Fluorescent Pseudomonads for Sugarcane Red Rot Suppression and Enhanced Yield Under Field Conditions</v>
+        <v>Physiology and dinitrogen fixation of A cetobacter diazotrophicus</v>
       </c>
       <c r="E125" t="str">
-        <v>Uso de Pseudomonas fluorescens para controle de doenças em cana-de-açúcar</v>
+        <v>N2-dependent growth; N2-fixation, in sugar cane; Acetobacter diazotrophicus</v>
       </c>
       <c r="F125">
-        <v>2003</v>
+        <v>1991</v>
       </c>
       <c r="G125" t="str">
         <v>N/A</v>
       </c>
       <c r="H125" t="str">
-        <v>Cana-de-açúcar, resistência sistêmica induzida, promoção de crescimento, Pseudomonas fluorescens, doença da rota vermelha</v>
+        <v>N2-dependent growth, N2-fixation, sugar cane, Acetobacter diazotrophicus</v>
       </c>
       <c r="I125" t="str">
-        <v>O estudo avaliou a eficácia de Pseudomonas fluorescens em controlar a doença da rota vermelha em cana-de-açúcar. As bactérias foram isoladas da rizosfera da cana-de-açúcar e formuladas em talco. A aplicação das bactérias reduziu a incidência da doença e melhorou a produção de cana-de-açúcar.</v>
+        <v>O artigo descreve as características fisiológicas de Acetobacter diazotrophicus, um diazotrófico isolado de raízes de cana-de-açúcar. O bactério é capaz de crescer em pH 3,0 e apresenta alta atividade de nitrogenase até pH 2,5. A extração de oxidação de glicose seguida pela formação de ácido gluconico é necessária para iniciar o crescimento logarítmico, que ocorre com N2 como fonte de nitrogênio.</v>
       </c>
       <c r="J125" t="str">
         <v>Artigo científico</v>
       </c>
       <c r="K125" t="str">
-        <v>Tamil Nadu Agricultural University</v>
+        <v>FEMS Microbiology Letters</v>
       </c>
       <c r="L125" t="str">
-        <v>Departamento de Patologia Vegetal, Universidade Agrícola de Tamil Nadu</v>
+        <v>CNPBS/EMBRAPA</v>
       </c>
       <c r="M125" t="str">
-        <v>Coimbatore, Índia</v>
+        <v>Seropédica, Rio de Janeiro, Brasil</v>
       </c>
       <c r="N125" t="str">
-        <v>Pesquisa</v>
+        <v>Estudo de caso</v>
       </c>
       <c r="O125" t="str">
-        <v>Vol. 5 (l&amp;2)</v>
+        <v>FEMS Microbiology Letters</v>
       </c>
       <c r="P125" t="str">
         <v>N/A</v>
       </c>
       <c r="Q125">
-        <v>5</v>
-      </c>
-      <c r="R125" t="str">
-        <v>l&amp;2</v>
+        <v>77</v>
+      </c>
+      <c r="R125">
+        <v>1</v>
       </c>
       <c r="S125" t="str">
-        <v>37-43</v>
+        <v>67-72</v>
       </c>
       <c r="T125" t="str">
         <v>N/A</v>
@@ -9236,28 +9239,28 @@
         <v>N/A</v>
       </c>
       <c r="W125" t="str">
-        <v>Talc Formulated Fluorescent Pseudomonads_bioinsumos.pdf</v>
+        <v>Physiology and dinitrogen fixation of A cetobacter diazotrophicus_bioinsumos.pdf</v>
       </c>
       <c r="Z125" t="str">
-        <v>N/A</v>
+        <v>O solo da região de cultivo da cana-de-açúcar é caracterizado por pH ácido, com valores entre 3,0 e 5,5. A região é localizada no Brasil, mais especificamente no estado do Rio de Janeiro.</v>
       </c>
       <c r="AA125" t="str">
-        <v>N/A</v>
+        <v>Cromatografia gasosa, Espectrometria de massa, Análise de variância (ANOVA)</v>
       </c>
       <c r="AB125" t="str">
-        <v>N/A</v>
+        <v>Nitrogênio, Fósforo, Potássio</v>
       </c>
       <c r="AC125" t="str">
-        <v>N/A</v>
+        <v>Fertilização de cobertura, Adubação foliar, Fertirrigação</v>
       </c>
       <c r="AD125" t="str">
-        <v>N/A</v>
+        <v>Cereais, Leguminosas, Hortaliças, Frutíferas</v>
       </c>
       <c r="AE125" t="str">
-        <v>N/A</v>
+        <v>Cana-de-açúcar</v>
       </c>
       <c r="AF125" t="str">
-        <v>Aprovado: Avalia a eficácia de Pseudomonas fluorescens em controlar a doença da rota vermelha em cana-de-açúcar.</v>
+        <v>Aprovado: Detalha as características fisiológicas de Acetobacter diazotrophicus e sua capacidade de fixação de nitrogênio.</v>
       </c>
       <c r="AG125" t="b">
         <v>1</v>
@@ -9271,28 +9274,34 @@
     </row>
     <row r="126">
       <c r="C126" t="str">
-        <v>K. HARI e T.R. SRINIVASAN</v>
+        <v>N. SenthiP, T. Raguchander, R. Viswanathan e R. Samiyappan</v>
       </c>
       <c r="D126" t="str">
-        <v>Response of Sugarcane Varieties to Application of Nitrogen Fixing Bacteria under Different Nitrogen Levels</v>
+        <v>Sugarcane Talc Formulated. Fluorescent Pseudomonads for Sugarcane Red Rot Suppression and Enhanced Yield Under Field Conditions</v>
       </c>
       <c r="E126" t="str">
-        <v>Efeito da aplicação de bactérias fixadoras de nitrogênio em variedades de cana-de-açúcar sob diferentes níveis de nitrogênio</v>
+        <v>Uso de Pseudomonas fluorescens para controle de doenças em cana-de-açúcar</v>
       </c>
       <c r="F126">
-        <v>2005</v>
+        <v>2003</v>
+      </c>
+      <c r="G126" t="str">
+        <v>N/A</v>
       </c>
       <c r="H126" t="str">
-        <v>cana-de-açúcar, biofertilizantes, Azotobacter, Azospirillum e Gluconacetobacter, bactérias fixadoras de nitrogênio</v>
+        <v>Cana-de-açúcar, resistência sistêmica induzida, promoção de crescimento, Pseudomonas fluorescens, doença da rota vermelha</v>
       </c>
       <c r="I126" t="str">
-        <v>O estudo avaliou a resposta de variedades de cana-de-açúcar à aplicação de Azotobacter, Azospirillum e Gluconacetobacter sob diferentes níveis de nitrogênio.</v>
+        <v>O estudo avaliou a eficácia de Pseudomonas fluorescens em controlar a doença da rota vermelha em cana-de-açúcar. As bactérias foram isoladas da rizosfera da cana-de-açúcar e formuladas em talco. A aplicação das bactérias reduziu a incidência da doença e melhorou a produção de cana-de-açúcar.</v>
       </c>
       <c r="J126" t="str">
         <v>Artigo científico</v>
       </c>
+      <c r="K126" t="str">
+        <v>Tamil Nadu Agricultural University</v>
+      </c>
       <c r="L126" t="str">
-        <v>Sugarcane Breeding Institute, ICAR, Coimbatore</v>
+        <v>Departamento de Patologia Vegetal, Universidade Agrícola de Tamil Nadu</v>
       </c>
       <c r="M126" t="str">
         <v>Coimbatore, Índia</v>
@@ -9300,14 +9309,32 @@
       <c r="N126" t="str">
         <v>Pesquisa</v>
       </c>
+      <c r="O126" t="str">
+        <v>Vol. 5 (l&amp;2)</v>
+      </c>
+      <c r="P126" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="Q126">
+        <v>5</v>
+      </c>
+      <c r="R126" t="str">
+        <v>l&amp;2</v>
+      </c>
       <c r="S126" t="str">
-        <v>28-31</v>
+        <v>37-43</v>
+      </c>
+      <c r="T126" t="str">
+        <v>N/A</v>
       </c>
       <c r="U126" t="str">
         <v>N/A</v>
       </c>
+      <c r="V126" t="str">
+        <v>N/A</v>
+      </c>
       <c r="W126" t="str">
-        <v>Response of sugarcane varieties to application of nitrogen fixing_bioinsumos.pdf</v>
+        <v>Talc Formulated Fluorescent Pseudomonads_bioinsumos.pdf</v>
       </c>
       <c r="Z126" t="str">
         <v>N/A</v>
@@ -9328,7 +9355,7 @@
         <v>N/A</v>
       </c>
       <c r="AF126" t="str">
-        <v>Aprovado: Avalia a eficácia de Azospirillum no controle de fungos em cana-de-açúcar.</v>
+        <v>Aprovado: Avalia a eficácia de Pseudomonas fluorescens em controlar a doença da rota vermelha em cana-de-açúcar.</v>
       </c>
       <c r="AG126" t="b">
         <v>1</v>
@@ -9342,204 +9369,147 @@
     </row>
     <row r="127">
       <c r="C127" t="str">
-        <v>Roberto Batista Marques Júnior, Luciano Pasqualoto Canellas, Lúcia Gracinda da Silva, Fábio Lopes Olivares</v>
+        <v>K. HARI e T.R. SRINIVASAN</v>
       </c>
       <c r="D127" t="str">
-        <v>PROMOÇÃO DE ENRAIZAMENTO DE MICROTOLETES DE CANA-DE-AÇÚCAR PELO USO CONJUNTO DE SUBSTÂNCIAS HÚMICAS E BACTÉRIAS DIAZOTRÓFICAS ENDOFÍTICAS</v>
+        <v>Response of Sugarcane Varieties to Application of Nitrogen Fixing Bacteria under Different Nitrogen Levels</v>
       </c>
       <c r="E127" t="str">
-        <v>ROOTING OF MICRO SEED PIECES BY COMBINED USE OF HUMIC SUBSTANCES AND ENDOPHYTIC DIAZOTROPHIC BACTERIA IN SUGAR CANE</v>
-      </c>
-      <c r="F127" t="str">
-        <v>2008</v>
-      </c>
-      <c r="G127" t="str">
-        <v/>
+        <v>Efeito da aplicação de bactérias fixadoras de nitrogênio em variedades de cana-de-açúcar sob diferentes níveis de nitrogênio</v>
+      </c>
+      <c r="F127">
+        <v>2005</v>
       </c>
       <c r="H127" t="str">
-        <v>Herbaspirillum seropedicae, termoterapia, ácidos húmicos</v>
+        <v>cana-de-açúcar, biofertilizantes, Azotobacter, Azospirillum e Gluconacetobacter, bactérias fixadoras de nitrogênio</v>
       </c>
       <c r="I127" t="str">
-        <v>Além do fornecimento direto de nutrientes por meio da mineralização da matéria orgânica ou pela fixação biológica de N 2, as substâncias húmicas e as bactérias diazotróficas endofíticas podem afetar diretamente o metabolismo vegetal, modificando o padrão de crescimento e desenvolvimento das plantas.</v>
+        <v>O estudo avaliou a resposta de variedades de cana-de-açúcar à aplicação de Azotobacter, Azospirillum e Gluconacetobacter sob diferentes níveis de nitrogênio.</v>
       </c>
       <c r="J127" t="str">
         <v>Artigo científico</v>
       </c>
-      <c r="K127" t="str">
-        <v/>
-      </c>
       <c r="L127" t="str">
-        <v>Universidade Estadual do Norte Fluminense - Darcy Ribeiro</v>
+        <v>Sugarcane Breeding Institute, ICAR, Coimbatore</v>
       </c>
       <c r="M127" t="str">
-        <v>Campos dos Goytacazes (RJ)</v>
+        <v>Coimbatore, Índia</v>
       </c>
       <c r="N127" t="str">
-        <v>Tese de Mestrado</v>
-      </c>
-      <c r="O127" t="str">
-        <v>Revista Brasileira de Ciência do Solo</v>
-      </c>
-      <c r="P127" t="str">
-        <v/>
-      </c>
-      <c r="Q127" t="str">
-        <v>32</v>
-      </c>
-      <c r="R127" t="str">
-        <v/>
+        <v>Pesquisa</v>
       </c>
       <c r="S127" t="str">
-        <v>1121-1128</v>
-      </c>
-      <c r="T127" t="str">
-        <v/>
+        <v>28-31</v>
       </c>
       <c r="U127" t="str">
         <v>N/A</v>
       </c>
-      <c r="V127" t="str">
-        <v/>
-      </c>
       <c r="W127" t="str">
-        <v>ROOTING OF MICRO SEED PIECES BY COMBINED USE_bioinsumos.pdf</v>
+        <v>Response of sugarcane varieties to application of nitrogen fixing_bioinsumos.pdf</v>
       </c>
       <c r="Z127" t="str">
         <v>N/A</v>
       </c>
       <c r="AA127" t="str">
-        <v>Cromatografia gasosa, Espectrometria de massa, Análise de variância (ANOVA)</v>
+        <v>N/A</v>
       </c>
       <c r="AB127" t="str">
-        <v>Nitrogênio, Fósforo, Potássio, Boro</v>
+        <v>N/A</v>
       </c>
       <c r="AC127" t="str">
-        <v>Fertilização de cobertura, Adubação foliar, Fertirrigação</v>
+        <v>N/A</v>
       </c>
       <c r="AD127" t="str">
-        <v>Cereais, Leguminosas, Hortaliças, Frutíferas</v>
+        <v>N/A</v>
       </c>
       <c r="AE127" t="str">
-        <v>Cana-de-açúcar</v>
+        <v>N/A</v>
       </c>
       <c r="AF127" t="str">
-        <v>Aprovado: Detalha uma nova técnica de promoção de enraizamento de microtoletes de cana-de-açúcar utilizando substâncias húmicas e bactérias diazotróficas endofíticas.</v>
-      </c>
-      <c r="AG127" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="AH127" t="str">
-        <v>FALSE</v>
+        <v>Aprovado: Avalia a eficácia de Azospirillum no controle de fungos em cana-de-açúcar.</v>
+      </c>
+      <c r="AG127" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH127" t="b">
+        <v>0</v>
       </c>
       <c r="AJ127" t="str">
         <v>BIOINSUMOS</v>
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="str">
-        <v/>
-      </c>
-      <c r="B128" t="str">
-        <v/>
-      </c>
       <c r="C128" t="str">
-        <v>M.P. Stephan, M. Oliveira, K.R.S. Teixeira, G. Martinez-Drets e J. D/Sbereiner</v>
+        <v>Roberto Batista Marques Júnior, Luciano Pasqualoto Canellas, Lúcia Gracinda da Silva, Fábio Lopes Olivares</v>
       </c>
       <c r="D128" t="str">
-        <v>Physiology and dinitrogen fixation of A cetobacter diazotrophicus</v>
+        <v>PROMOÇÃO DE ENRAIZAMENTO DE MICROTOLETES DE CANA-DE-AÇÚCAR PELO USO CONJUNTO DE SUBSTÂNCIAS HÚMICAS E BACTÉRIAS DIAZOTRÓFICAS ENDOFÍTICAS</v>
       </c>
       <c r="E128" t="str">
-        <v>Estudo sobre a fixação de nitrogênio e características fisiológicas de Acetobacter diazotrophicus</v>
-      </c>
-      <c r="F128" t="str">
-        <v>1991</v>
-      </c>
-      <c r="G128" t="str">
-        <v/>
+        <v>ROOTING OF MICRO SEED PIECES BY COMBINED USE OF HUMIC SUBSTANCES AND ENDOPHYTIC DIAZOTROPHIC BACTERIA IN SUGAR CANE</v>
+      </c>
+      <c r="F128">
+        <v>2008</v>
       </c>
       <c r="H128" t="str">
-        <v>N2-dependent growth, N2-fixation, in sugar cane, Acetobacter diazotrophicus</v>
+        <v>Herbaspirillum seropedicae, termoterapia, ácidos húmicos</v>
       </c>
       <c r="I128" t="str">
-        <v>O artigo descreve as características fisiológicas e a fixação de nitrogênio de Acetobacter diazotrophicus, um bactério isolado de raízes de cana-de-açúcar.</v>
+        <v>Além do fornecimento direto de nutrientes por meio da mineralização da matéria orgânica ou pela fixação biológica de N 2, as substâncias húmicas e as bactérias diazotróficas endofíticas podem afetar diretamente o metabolismo vegetal, modificando o padrão de crescimento e desenvolvimento das plantas.</v>
       </c>
       <c r="J128" t="str">
         <v>Artigo científico</v>
       </c>
-      <c r="K128" t="str">
-        <v>FEMS Microbiology Letters</v>
-      </c>
       <c r="L128" t="str">
-        <v>CNPBS/EMBRAPA</v>
+        <v>Universidade Estadual do Norte Fluminense - Darcy Ribeiro</v>
       </c>
       <c r="M128" t="str">
-        <v>Seropédica, Rio de Janeiro, Brasil</v>
+        <v>Campos dos Goytacazes (RJ)</v>
       </c>
       <c r="N128" t="str">
-        <v>Estudo de caso</v>
+        <v>Tese de Mestrado</v>
       </c>
       <c r="O128" t="str">
-        <v>FEMS Microbiology Letters</v>
-      </c>
-      <c r="P128" t="str">
-        <v/>
-      </c>
-      <c r="Q128" t="str">
-        <v>77</v>
-      </c>
-      <c r="R128" t="str">
-        <v>1</v>
+        <v>Revista Brasileira de Ciência do Solo</v>
+      </c>
+      <c r="Q128">
+        <v>32</v>
       </c>
       <c r="S128" t="str">
-        <v>67-72</v>
-      </c>
-      <c r="T128" t="str">
-        <v/>
+        <v>1121-1128</v>
       </c>
       <c r="U128" t="str">
         <v>N/A</v>
       </c>
-      <c r="V128" t="str">
-        <v/>
-      </c>
       <c r="W128" t="str">
-        <v>Physiology and dinitrogen fixation of A cetobacter diazotrophicus_bioinsumos.pdf</v>
-      </c>
-      <c r="X128" t="str">
-        <v/>
-      </c>
-      <c r="Y128" t="str">
-        <v/>
+        <v>ROOTING OF MICRO SEED PIECES BY COMBINED USE_bioinsumos.pdf</v>
       </c>
       <c r="Z128" t="str">
         <v>N/A</v>
       </c>
       <c r="AA128" t="str">
-        <v>PCR, Sequenciamento, Microscopia, Ensaios em vasos</v>
+        <v>Cromatografia gasosa, Espectrometria de massa, Análise de variância (ANOVA)</v>
       </c>
       <c r="AB128" t="str">
-        <v>Acetobacter diazotrophicus</v>
+        <v>Nitrogênio, Fósforo, Potássio, Boro</v>
       </c>
       <c r="AC128" t="str">
-        <v>Inoculação de sementes</v>
+        <v>Fertilização de cobertura, Adubação foliar, Fertirrigação</v>
       </c>
       <c r="AD128" t="str">
+        <v>Cereais, Leguminosas, Hortaliças, Frutíferas</v>
+      </c>
+      <c r="AE128" t="str">
         <v>Cana-de-açúcar</v>
       </c>
-      <c r="AE128" t="str">
-        <v>Acetobacter diazotrophicus</v>
-      </c>
       <c r="AF128" t="str">
-        <v>Aprovado: Avalia a eficácia de Acetobacter diazotrophicus na fixação de nitrogênio em cana-de-açúcar.</v>
-      </c>
-      <c r="AG128" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="AH128" t="str">
-        <v>FALSE</v>
-      </c>
-      <c r="AI128" t="str">
-        <v/>
+        <v>Aprovado: Detalha uma nova técnica de promoção de enraizamento de microtoletes de cana-de-açúcar utilizando substâncias húmicas e bactérias diazotróficas endofíticas.</v>
+      </c>
+      <c r="AG128" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH128" t="b">
+        <v>0</v>
       </c>
       <c r="AJ128" t="str">
         <v>BIOINSUMOS</v>

</xml_diff>

<commit_message>
Correcao de classificação, marcação de cieto e curadoria
</commit_message>
<xml_diff>
--- a/squad1/ciento/api-cientometria/Consolidado - Respostas Gerais.xlsx
+++ b/squad1/ciento/api-cientometria/Consolidado - Respostas Gerais.xlsx
@@ -596,7 +596,7 @@
         <v>1</v>
       </c>
       <c r="AJ2" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="3">
@@ -670,7 +670,7 @@
         <v>1</v>
       </c>
       <c r="AJ3" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="4">
@@ -744,7 +744,7 @@
         <v>0</v>
       </c>
       <c r="AJ4" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="5">
@@ -818,7 +818,7 @@
         <v>0</v>
       </c>
       <c r="AJ5" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="6">
@@ -892,7 +892,7 @@
         <v>0</v>
       </c>
       <c r="AJ6" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="7">
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
       <c r="AJ7" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="8">
@@ -1025,7 +1025,7 @@
         <v>0</v>
       </c>
       <c r="AJ8" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="9">
@@ -1096,7 +1096,7 @@
         <v>0</v>
       </c>
       <c r="AJ9" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="10">
@@ -1170,7 +1170,7 @@
         <v>0</v>
       </c>
       <c r="AJ10" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="11">
@@ -1238,7 +1238,7 @@
         <v>0</v>
       </c>
       <c r="AJ11" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="12">
@@ -1309,7 +1309,7 @@
         <v>0</v>
       </c>
       <c r="AJ12" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="13">
@@ -1377,7 +1377,7 @@
         <v>0</v>
       </c>
       <c r="AJ13" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="14">
@@ -1448,7 +1448,7 @@
         <v>0</v>
       </c>
       <c r="AJ14" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="15">
@@ -1510,7 +1510,7 @@
         <v>0</v>
       </c>
       <c r="AJ15" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="16">
@@ -1584,7 +1584,7 @@
         <v>0</v>
       </c>
       <c r="AJ16" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="17">
@@ -1655,7 +1655,7 @@
         <v>0</v>
       </c>
       <c r="AJ17" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="18">
@@ -1729,7 +1729,7 @@
         <v>0</v>
       </c>
       <c r="AJ18" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="19">
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="AJ19" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="20">
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="AJ20" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="21">
@@ -1945,7 +1945,7 @@
         <v>0</v>
       </c>
       <c r="AJ21" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="22">
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="AJ22" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="23">
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="AJ23" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="24">
@@ -2143,7 +2143,7 @@
         <v>0</v>
       </c>
       <c r="AJ24" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="25">
@@ -2217,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="AJ25" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="26">
@@ -2282,7 +2282,7 @@
         <v>0</v>
       </c>
       <c r="AJ26" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="27">
@@ -2353,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="AJ27" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="28">
@@ -2427,7 +2427,7 @@
         <v>0</v>
       </c>
       <c r="AJ28" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="29">
@@ -2501,7 +2501,7 @@
         <v>0</v>
       </c>
       <c r="AJ29" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="30">
@@ -2569,7 +2569,7 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="31">
@@ -2643,7 +2643,7 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="32">
@@ -2717,7 +2717,7 @@
         <v>0</v>
       </c>
       <c r="AJ32" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="33">
@@ -2791,7 +2791,7 @@
         <v>0</v>
       </c>
       <c r="AJ33" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="34">
@@ -2865,7 +2865,7 @@
         <v>0</v>
       </c>
       <c r="AJ34" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="35">
@@ -2939,7 +2939,7 @@
         <v>0</v>
       </c>
       <c r="AJ35" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="36">
@@ -3007,7 +3007,7 @@
         <v>0</v>
       </c>
       <c r="AJ36" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="37">
@@ -3078,7 +3078,7 @@
         <v>0</v>
       </c>
       <c r="AJ37" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="38">
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="AJ38" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="39">
@@ -3220,7 +3220,7 @@
         <v>0</v>
       </c>
       <c r="AJ39" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="40">
@@ -3291,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="AJ40" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="41">
@@ -3365,7 +3365,7 @@
         <v>0</v>
       </c>
       <c r="AJ41" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="42">
@@ -3436,7 +3436,7 @@
         <v>0</v>
       </c>
       <c r="AJ42" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="43">
@@ -3507,7 +3507,7 @@
         <v>0</v>
       </c>
       <c r="AJ43" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="44">
@@ -3581,7 +3581,7 @@
         <v>0</v>
       </c>
       <c r="AJ44" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="45">
@@ -3649,7 +3649,7 @@
         <v>0</v>
       </c>
       <c r="AJ45" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="46">
@@ -3720,7 +3720,7 @@
         <v>0</v>
       </c>
       <c r="AJ46" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="47">
@@ -3791,7 +3791,7 @@
         <v>0</v>
       </c>
       <c r="AJ47" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="48">
@@ -3865,7 +3865,7 @@
         <v>0</v>
       </c>
       <c r="AJ48" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="49">
@@ -3939,7 +3939,7 @@
         <v>0</v>
       </c>
       <c r="AJ49" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="50">
@@ -4010,7 +4010,7 @@
         <v>0</v>
       </c>
       <c r="AJ50" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="51">
@@ -4072,7 +4072,7 @@
         <v>0</v>
       </c>
       <c r="AJ51" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="52">
@@ -4146,7 +4146,7 @@
         <v>0</v>
       </c>
       <c r="AJ52" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="53">
@@ -4220,7 +4220,7 @@
         <v>0</v>
       </c>
       <c r="AJ53" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="54">
@@ -4294,7 +4294,7 @@
         <v>0</v>
       </c>
       <c r="AJ54" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="55">
@@ -4368,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="AJ55" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="56">
@@ -4442,7 +4442,7 @@
         <v>0</v>
       </c>
       <c r="AJ56" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="57">
@@ -4516,7 +4516,7 @@
         <v>0</v>
       </c>
       <c r="AJ57" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="58">
@@ -4581,7 +4581,7 @@
         <v>0</v>
       </c>
       <c r="AJ58" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="59">
@@ -4652,7 +4652,7 @@
         <v>0</v>
       </c>
       <c r="AJ59" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="60">
@@ -4726,7 +4726,7 @@
         <v>0</v>
       </c>
       <c r="AJ60" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="61">
@@ -4788,7 +4788,7 @@
         <v>0</v>
       </c>
       <c r="AJ61" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="62">
@@ -4862,7 +4862,7 @@
         <v>0</v>
       </c>
       <c r="AJ62" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="63">
@@ -4936,7 +4936,7 @@
         <v>0</v>
       </c>
       <c r="AJ63" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="64">
@@ -5007,7 +5007,7 @@
         <v>0</v>
       </c>
       <c r="AJ64" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="65">
@@ -5081,7 +5081,7 @@
         <v>0</v>
       </c>
       <c r="AJ65" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="66">
@@ -5155,7 +5155,7 @@
         <v>0</v>
       </c>
       <c r="AJ66" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="67">
@@ -5229,7 +5229,7 @@
         <v>0</v>
       </c>
       <c r="AJ67" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="68">
@@ -5300,7 +5300,7 @@
         <v>0</v>
       </c>
       <c r="AJ68" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="69">
@@ -5374,7 +5374,7 @@
         <v>0</v>
       </c>
       <c r="AJ69" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="70">
@@ -5448,7 +5448,7 @@
         <v>0</v>
       </c>
       <c r="AJ70" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="71">
@@ -5522,7 +5522,7 @@
         <v>0</v>
       </c>
       <c r="AJ71" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="72">
@@ -5593,7 +5593,7 @@
         <v>0</v>
       </c>
       <c r="AJ72" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="73">
@@ -5667,7 +5667,7 @@
         <v>0</v>
       </c>
       <c r="AJ73" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="74">
@@ -5738,7 +5738,7 @@
         <v>0</v>
       </c>
       <c r="AJ74" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="75">
@@ -5812,7 +5812,7 @@
         <v>0</v>
       </c>
       <c r="AJ75" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="76">
@@ -5880,7 +5880,7 @@
         <v>0</v>
       </c>
       <c r="AJ76" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="77">
@@ -5951,7 +5951,7 @@
         <v>0</v>
       </c>
       <c r="AJ77" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="78">
@@ -6022,7 +6022,7 @@
         <v>0</v>
       </c>
       <c r="AJ78" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="79">
@@ -6096,7 +6096,7 @@
         <v>0</v>
       </c>
       <c r="AJ79" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="80">
@@ -6167,7 +6167,7 @@
         <v>0</v>
       </c>
       <c r="AJ80" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="81">
@@ -6229,7 +6229,7 @@
         <v>0</v>
       </c>
       <c r="AJ81" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="82">
@@ -6300,7 +6300,7 @@
         <v>0</v>
       </c>
       <c r="AJ82" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="83">
@@ -6362,7 +6362,7 @@
         <v>0</v>
       </c>
       <c r="AJ83" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="84">
@@ -6418,7 +6418,7 @@
         <v>0</v>
       </c>
       <c r="AJ84" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="85">
@@ -6492,7 +6492,7 @@
         <v>0</v>
       </c>
       <c r="AJ85" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="86">
@@ -6551,7 +6551,7 @@
         <v>0</v>
       </c>
       <c r="AJ86" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="87">
@@ -6610,7 +6610,7 @@
         <v>0</v>
       </c>
       <c r="AJ87" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="88">
@@ -6684,7 +6684,7 @@
         <v>0</v>
       </c>
       <c r="AJ88" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="89">
@@ -6752,7 +6752,7 @@
         <v>0</v>
       </c>
       <c r="AJ89" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="90">
@@ -6808,7 +6808,7 @@
         <v>0</v>
       </c>
       <c r="AJ90" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="91">
@@ -6879,7 +6879,7 @@
         <v>0</v>
       </c>
       <c r="AJ91" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="92">
@@ -6950,7 +6950,7 @@
         <v>0</v>
       </c>
       <c r="AJ92" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="93">
@@ -7024,7 +7024,7 @@
         <v>0</v>
       </c>
       <c r="AJ93" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="94">
@@ -7098,7 +7098,7 @@
         <v>0</v>
       </c>
       <c r="AJ94" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="95">
@@ -7169,7 +7169,7 @@
         <v>0</v>
       </c>
       <c r="AJ95" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="96">
@@ -7231,7 +7231,7 @@
         <v>0</v>
       </c>
       <c r="AJ96" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="97">
@@ -7296,7 +7296,7 @@
         <v>0</v>
       </c>
       <c r="AJ97" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="98">
@@ -7358,7 +7358,7 @@
         <v>0</v>
       </c>
       <c r="AJ98" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="99">
@@ -7417,7 +7417,7 @@
         <v>0</v>
       </c>
       <c r="AJ99" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="100">
@@ -7482,7 +7482,7 @@
         <v>0</v>
       </c>
       <c r="AJ100" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="101">
@@ -7550,7 +7550,7 @@
         <v>0</v>
       </c>
       <c r="AJ101" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="102">
@@ -7624,7 +7624,7 @@
         <v>0</v>
       </c>
       <c r="AJ102" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="103">
@@ -7677,7 +7677,7 @@
         <v>0</v>
       </c>
       <c r="AJ103" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="104">
@@ -7739,7 +7739,7 @@
         <v>0</v>
       </c>
       <c r="AJ104" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="105">
@@ -7807,7 +7807,7 @@
         <v>0</v>
       </c>
       <c r="AJ105" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="106">
@@ -7869,7 +7869,7 @@
         <v>0</v>
       </c>
       <c r="AJ106" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="107">
@@ -7928,7 +7928,7 @@
         <v>0</v>
       </c>
       <c r="AJ107" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="108">
@@ -8002,7 +8002,7 @@
         <v>0</v>
       </c>
       <c r="AJ108" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="109">
@@ -8064,7 +8064,7 @@
         <v>0</v>
       </c>
       <c r="AJ109" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="110">
@@ -8126,7 +8126,7 @@
         <v>0</v>
       </c>
       <c r="AJ110" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="111">
@@ -8188,7 +8188,7 @@
         <v>0</v>
       </c>
       <c r="AJ111" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="112">
@@ -8250,7 +8250,7 @@
         <v>0</v>
       </c>
       <c r="AJ112" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="113">
@@ -8324,7 +8324,7 @@
         <v>0</v>
       </c>
       <c r="AJ113" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="114">
@@ -8383,7 +8383,7 @@
         <v>0</v>
       </c>
       <c r="AJ114" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="115">
@@ -8454,7 +8454,7 @@
         <v>0</v>
       </c>
       <c r="AJ115" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="116">
@@ -8522,7 +8522,7 @@
         <v>0</v>
       </c>
       <c r="AJ116" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="117">
@@ -8581,7 +8581,7 @@
         <v>0</v>
       </c>
       <c r="AJ117" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="118">
@@ -8643,7 +8643,7 @@
         <v>0</v>
       </c>
       <c r="AJ118" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="119">
@@ -8702,7 +8702,7 @@
         <v>0</v>
       </c>
       <c r="AJ119" t="str">
-        <v>MANEJO DE NUTRIENTES E AGUA</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="120">
@@ -8806,7 +8806,7 @@
         <v>0</v>
       </c>
       <c r="AJ120" t="str">
-        <v>MANEJO ECOFISIOLÓGICO E NUTRICIONAL DA CITRICULTURA DE ALTA PERFORMANCE</v>
+        <v>citros e cana</v>
       </c>
     </row>
     <row r="121">
@@ -8901,7 +8901,7 @@
         <v>0</v>
       </c>
       <c r="AJ121" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
     <row r="122">
@@ -9094,7 +9094,7 @@
         <v>0</v>
       </c>
       <c r="AJ123" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
     <row r="124">
@@ -9174,7 +9174,7 @@
         <v>0</v>
       </c>
       <c r="AJ124" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
     <row r="125">
@@ -9269,7 +9269,7 @@
         <v>0</v>
       </c>
       <c r="AJ125" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
     <row r="126">
@@ -9364,7 +9364,7 @@
         <v>0</v>
       </c>
       <c r="AJ126" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
     <row r="127">
@@ -9435,7 +9435,7 @@
         <v>0</v>
       </c>
       <c r="AJ127" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
     <row r="128">
@@ -9512,7 +9512,7 @@
         <v>0</v>
       </c>
       <c r="AJ128" t="str">
-        <v>BIOINSUMOS</v>
+        <v>solos</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
arrumando o manual insert
</commit_message>
<xml_diff>
--- a/squad1/ciento/api-cientometria/Consolidado - Respostas Gerais.xlsx
+++ b/squad1/ciento/api-cientometria/Consolidado - Respostas Gerais.xlsx
@@ -8713,7 +8713,7 @@
         <v>izaias silva</v>
       </c>
       <c r="C120" t="str">
-        <v>N/A</v>
+        <v xml:space="preserve">ERRO: Erro na API do LLM: </v>
       </c>
       <c r="D120" t="str">
         <v>N/A</v>
@@ -8794,13 +8794,13 @@
         <v>N/A</v>
       </c>
       <c r="AF120" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="AG120" t="b">
-        <v>0</v>
-      </c>
-      <c r="AH120" t="b">
-        <v>1</v>
+        <v xml:space="preserve">Erro na análise: ERRO: Erro na API do LLM: </v>
+      </c>
+      <c r="AG120" t="str">
+        <v>FALSE</v>
+      </c>
+      <c r="AH120" t="str">
+        <v>TRUE</v>
       </c>
       <c r="AI120" t="b">
         <v>0</v>

</xml_diff>